<commit_message>
LOC Public Plugins Snapshot 2026-09-14
</commit_message>
<xml_diff>
--- a/loc-data-model-ext/templates/bulk_import_template.xlsx
+++ b/loc-data-model-ext/templates/bulk_import_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bhoffman/D/loc_archivesspace/loc-data-model-ext/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDFB027-7F44-014D-B68C-AB7149D40ABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA2A0CDD-5443-2646-B047-1B3051B81CFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="27200" windowHeight="16520" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Documentation" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="564">
   <si>
     <t>This is the template for importing archival objects using the bulk_import ("Load SpreadSheet").  You may replace this line with something of your choosing after you've copied the file for your use.</t>
   </si>
@@ -1632,6 +1632,9 @@
     <t>ead_dao_type</t>
   </si>
   <si>
+    <t>ead_dao_other_type</t>
+  </si>
+  <si>
     <t>descriptive_note</t>
   </si>
   <si>
@@ -1650,7 +1653,82 @@
     <t>additional_identifier_2</t>
   </si>
   <si>
-    <t>other_ead_dao_type</t>
+    <t>Note with Type=Other Finding Aid Note</t>
+  </si>
+  <si>
+    <t>Publish (true/false) Other Finding Aid Note</t>
+  </si>
+  <si>
+    <t>Label Other Finding Aid Note</t>
+  </si>
+  <si>
+    <t>Note with Type=Other Finding Aid Note (2)</t>
+  </si>
+  <si>
+    <t>Publish (true/false) Other Finding Aid Note (2)</t>
+  </si>
+  <si>
+    <t>Label Other Finding Aid Note (2)</t>
+  </si>
+  <si>
+    <t>Note with Type=Other Finding Aid Note (3)</t>
+  </si>
+  <si>
+    <t>Publish (true/false) Other Finding Aid Note (3)</t>
+  </si>
+  <si>
+    <t>Label Other Finding Aid Note (3)</t>
+  </si>
+  <si>
+    <t>n_otherfindaid</t>
+  </si>
+  <si>
+    <t>p_otherfindaid</t>
+  </si>
+  <si>
+    <t>l_otherfindaid</t>
+  </si>
+  <si>
+    <t>n_otherfindaid_2</t>
+  </si>
+  <si>
+    <t>p_otherfindaid_2</t>
+  </si>
+  <si>
+    <t>l_otherfindaid_2</t>
+  </si>
+  <si>
+    <t>n_otherfindaid_3</t>
+  </si>
+  <si>
+    <t>p_otherfindaid_3</t>
+  </si>
+  <si>
+    <t>l_otherfindaid_3</t>
+  </si>
+  <si>
+    <t>Other Finding Aid Note</t>
+  </si>
+  <si>
+    <t>Publish Other Finding Aid Note?</t>
+  </si>
+  <si>
+    <t>Other Finding Aid Note 2</t>
+  </si>
+  <si>
+    <t>Publish Other Finding Aid Note 2?</t>
+  </si>
+  <si>
+    <t>Label Other Finding Aid Note 2</t>
+  </si>
+  <si>
+    <t>Other Finding Aid Note 3</t>
+  </si>
+  <si>
+    <t>Publish Other Finding Aid Note 3?</t>
+  </si>
+  <si>
+    <t>Label Other Finding Aid Note 3</t>
   </si>
 </sst>
 </file>
@@ -2609,7 +2687,7 @@
     <col min="187" max="1030" width="9.33203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:202" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:211" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2631,7 +2709,7 @@
       <c r="GA1" s="2"/>
       <c r="GD1" s="2"/>
     </row>
-    <row r="2" spans="1:202" ht="61" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:211" ht="61" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>1</v>
       </c>
@@ -3238,8 +3316,35 @@
       <c r="GT2" s="18" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:202" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="GU2" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="GV2" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="GW2" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="GX2" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="GY2" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="GZ2" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="HA2" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="HB2" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="HC2" s="18" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:211" ht="105.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="19" t="s">
         <v>15</v>
       </c>
@@ -3278,10 +3383,10 @@
         <v>26</v>
       </c>
       <c r="N3" s="20" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="O3" s="20" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="P3" s="23" t="s">
         <v>27</v>
@@ -3844,8 +3949,35 @@
       <c r="GT3" s="36" t="s">
         <v>519</v>
       </c>
-    </row>
-    <row r="4" spans="1:202" s="43" customFormat="1" ht="56.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="GU3" s="36" t="s">
+        <v>538</v>
+      </c>
+      <c r="GV3" s="36" t="s">
+        <v>539</v>
+      </c>
+      <c r="GW3" s="36" t="s">
+        <v>540</v>
+      </c>
+      <c r="GX3" s="36" t="s">
+        <v>541</v>
+      </c>
+      <c r="GY3" s="36" t="s">
+        <v>542</v>
+      </c>
+      <c r="GZ3" s="36" t="s">
+        <v>543</v>
+      </c>
+      <c r="HA3" s="36" t="s">
+        <v>544</v>
+      </c>
+      <c r="HB3" s="36" t="s">
+        <v>545</v>
+      </c>
+      <c r="HC3" s="36" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="4" spans="1:211" s="43" customFormat="1" ht="56.25" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="37" t="s">
         <v>151</v>
       </c>
@@ -3886,10 +4018,10 @@
         <v>163</v>
       </c>
       <c r="N4" s="38" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="O4" s="38" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="P4" s="38" t="s">
         <v>164</v>
@@ -4111,13 +4243,13 @@
         <v>530</v>
       </c>
       <c r="CK4" s="38" t="s">
-        <v>537</v>
+        <v>531</v>
       </c>
       <c r="CL4" s="38" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="CM4" s="38" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="CN4" s="38" t="s">
         <v>235</v>
@@ -4452,8 +4584,35 @@
       <c r="GT4" s="38" t="s">
         <v>522</v>
       </c>
-    </row>
-    <row r="5" spans="1:202" ht="57" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="GU4" s="38" t="s">
+        <v>547</v>
+      </c>
+      <c r="GV4" s="38" t="s">
+        <v>548</v>
+      </c>
+      <c r="GW4" s="38" t="s">
+        <v>549</v>
+      </c>
+      <c r="GX4" s="38" t="s">
+        <v>550</v>
+      </c>
+      <c r="GY4" s="38" t="s">
+        <v>551</v>
+      </c>
+      <c r="GZ4" s="38" t="s">
+        <v>552</v>
+      </c>
+      <c r="HA4" s="38" t="s">
+        <v>553</v>
+      </c>
+      <c r="HB4" s="38" t="s">
+        <v>554</v>
+      </c>
+      <c r="HC4" s="38" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="5" spans="1:211" ht="57" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="44" t="s">
         <v>337</v>
       </c>
@@ -4494,10 +4653,10 @@
         <v>348</v>
       </c>
       <c r="N5" s="47" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="O5" s="47" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="P5" s="47" t="s">
         <v>5</v>
@@ -5060,12 +5219,40 @@
       <c r="GT5" s="47" t="s">
         <v>525</v>
       </c>
-    </row>
-    <row r="6" spans="1:202" ht="16" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="GU5" s="47" t="s">
+        <v>556</v>
+      </c>
+      <c r="GV5" s="47" t="s">
+        <v>557</v>
+      </c>
+      <c r="GW5" s="47" t="s">
+        <v>540</v>
+      </c>
+      <c r="GX5" s="47" t="s">
+        <v>558</v>
+      </c>
+      <c r="GY5" s="47" t="s">
+        <v>559</v>
+      </c>
+      <c r="GZ5" s="47" t="s">
+        <v>560</v>
+      </c>
+      <c r="HA5" s="47" t="s">
+        <v>561</v>
+      </c>
+      <c r="HB5" s="47" t="s">
+        <v>562</v>
+      </c>
+      <c r="HC5" s="47" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="6" spans="1:211" ht="16" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="N6"/>
       <c r="BO6" s="51"/>
       <c r="BP6" s="2"/>
     </row>
-    <row r="7" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:211" x14ac:dyDescent="0.2">
       <c r="EE7" s="2"/>
       <c r="EH7" s="2"/>
       <c r="EN7" s="2"/>
@@ -5085,7 +5272,7 @@
       <c r="GA7" s="2"/>
       <c r="GD7" s="2"/>
     </row>
-    <row r="8" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:211" x14ac:dyDescent="0.2">
       <c r="EE8" s="2"/>
       <c r="EH8" s="2"/>
       <c r="EN8" s="2"/>
@@ -5105,7 +5292,7 @@
       <c r="GA8" s="2"/>
       <c r="GD8" s="2"/>
     </row>
-    <row r="9" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:211" x14ac:dyDescent="0.2">
       <c r="EE9" s="2"/>
       <c r="EH9" s="2"/>
       <c r="EN9" s="2"/>
@@ -5125,7 +5312,7 @@
       <c r="GA9" s="2"/>
       <c r="GD9" s="2"/>
     </row>
-    <row r="10" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:211" x14ac:dyDescent="0.2">
       <c r="EE10" s="2"/>
       <c r="EH10" s="2"/>
       <c r="EN10" s="2"/>
@@ -5145,7 +5332,7 @@
       <c r="GA10" s="2"/>
       <c r="GD10" s="2"/>
     </row>
-    <row r="11" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:211" x14ac:dyDescent="0.2">
       <c r="EE11" s="2"/>
       <c r="EH11" s="2"/>
       <c r="EN11" s="2"/>
@@ -5165,7 +5352,7 @@
       <c r="GA11" s="2"/>
       <c r="GD11" s="2"/>
     </row>
-    <row r="12" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:211" x14ac:dyDescent="0.2">
       <c r="EE12" s="2"/>
       <c r="EH12" s="2"/>
       <c r="EN12" s="2"/>
@@ -5185,7 +5372,7 @@
       <c r="GA12" s="2"/>
       <c r="GD12" s="2"/>
     </row>
-    <row r="13" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:211" x14ac:dyDescent="0.2">
       <c r="EE13" s="2"/>
       <c r="EH13" s="2"/>
       <c r="EN13" s="2"/>
@@ -5205,7 +5392,7 @@
       <c r="GA13" s="2"/>
       <c r="GD13" s="2"/>
     </row>
-    <row r="14" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:211" x14ac:dyDescent="0.2">
       <c r="EE14" s="2"/>
       <c r="EH14" s="2"/>
       <c r="EN14" s="2"/>
@@ -5225,7 +5412,7 @@
       <c r="GA14" s="2"/>
       <c r="GD14" s="2"/>
     </row>
-    <row r="15" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:211" x14ac:dyDescent="0.2">
       <c r="EE15" s="2"/>
       <c r="EH15" s="2"/>
       <c r="EN15" s="2"/>
@@ -5245,7 +5432,7 @@
       <c r="GA15" s="2"/>
       <c r="GD15" s="2"/>
     </row>
-    <row r="16" spans="1:202" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:211" x14ac:dyDescent="0.2">
       <c r="EE16" s="2"/>
       <c r="EH16" s="2"/>
       <c r="EN16" s="2"/>
@@ -25046,12 +25233,12 @@
       <c r="GD1005" s="2"/>
     </row>
   </sheetData>
-  <dataValidations count="10">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I6:I1005" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations count="13">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I7:I1005" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Class,Collection,File,Fonds,Item,Other Level,Record Group,Series,Sub-Fonds,Sub-Group,Sub-Series"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ6:BZ1005 L6:L1005 BN6:BN1000" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BZ6:BZ1005 BN6:BN1000 L7:L1005" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"FALSE,TRUE"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -25063,7 +25250,7 @@
       <formula1>1</formula1>
       <formula2>20</formula2>
     </dataValidation>
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="K6:K1005 S6:S1005 W6:W1005 EK6:EK1005 EN6:EN1005 ET6:ET1005 EW6:EW1005 EZ6:EZ1005 FC6:FC1005 FF6:FF1005 FI6:FI1005 FL6:FL1005 FO6:FO1005 FR6:FR1005 FU6:FU1005 FX6:FX1005 GA6:GA1005 GD6:GD1005 GG6:GG1005 GJ6:GJ1005 GM6:GM1005 GP6:GP1005 GS6:GS1005" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="S6:S1005 W6:W1005 EK6:EK1005 EN6:EN1005 ET6:ET1005 EW6:EW1005 EZ6:EZ1005 FC6:FC1005 FF6:FF1005 FI6:FI1005 FL6:FL1005 FO6:FO1005 FR6:FR1005 FU6:FU1005 FX6:FX1005 GA6:GA1005 GD6:GD1005 GG6:GG1005 GJ6:GJ1005 K7:K1005 GP6:GP9 GP11:GP1005 GM6:GM9 GM11:GM1005 GS6:GS9 GS11:GS1005 GY6 GV6 HB6" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"FALSE,TRUE"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -25087,6 +25274,15 @@
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="K6" xr:uid="{25A3DC01-9F94-BA4C-85FF-0D3305AF5415}">
+      <formula1>"FALSE,TRUE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L6" xr:uid="{15871CF9-9C5A-9543-BE1A-B37BEDDB6400}">
+      <formula1>"FALSE,TRUE"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I6" xr:uid="{B3EAE486-19C2-544F-BD56-7EF8950273B6}">
+      <formula1>"Class,Collection,File,Fonds,Item,Other Level,Record Group,Series,Sub-Fonds,Sub-Group,Sub-Series"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>